<commit_message>
Task #225: Smart G4 Import Phase 1 — Complete
Backend:
- phone_utils.py: Added clean_phone_for_import() and landline support in normalize_israeli_phone
- import_router.py: Full rewrite with HEADER_ALIASES smart column detection (exact→contains fallback),
  project structure cross-reference (building/unit matching with ambiguity handling), date parsing,
  expanded schema (phone_2, handover_date, unit_type), server-side unit_id validation on execute
- g4_template.xlsx: Regenerated with 12 columns

Frontend:
- G4ImportModal.js: Complete rewrite — detected columns banner, match status badges (matched/overwrite/
  not_found/building_not_found/ambiguous), filter buttons, adaptive table columns based on detected
  columns, summary bar with counts, execute sends only matched/overwrite rows with cross-reference IDs
- api.js: No changes needed — existing execute function passes rows correctly

Build verified, e2e test passed.
</commit_message>
<xml_diff>
--- a/backend/static/g4_template.xlsx
+++ b/backend/static/g4_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נתוני רוכשים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="G4 Import" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +28,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,8 +40,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="002563EB"/>
+        <bgColor rgb="002563EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,10 +54,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -69,7 +77,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,21 +444,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>בניין</t>
@@ -483,34 +494,49 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>מייל</t>
+          <t>אימייל</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>שם רוכש 2</t>
+          <t>שם נוסף</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ת"ז רוכש 2</t>
+          <t>ת"ז נוסף</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>טלפון נוסף</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>תאריך מסירה</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>אפיון דירה</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>בניין A</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>101</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -525,12 +551,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>050-1234567</t>
+          <t>0501234567</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>israel@email.com</t>
+          <t>test@email.com</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -541,82 +567,119 @@
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>987654321</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>0521234567</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>14/12/2024</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>דירה</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>בניין A</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>102</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>דוד כהן</t>
+          <t>משה כהן</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>111222333</t>
+          <t>234567890</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>052-9876543</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>david@email.com</t>
-        </is>
-      </c>
+          <t>0531234567</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>15/12/2024</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>מחיר למשתכן</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>בניין A</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>201</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>יעקב לוי</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>345678901</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0541234567</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>רחל לוי</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>444555666</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>054-5551234</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>456789012</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>דירה</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>